<commit_message>
Corregir escenario prudente: personal 2028 fijo y alza de alquiler
- Personal: 2027 y 2028 al nivel de 2026 +20% (91.559,58 EUR)
- Otros gastos: +5.000 EUR de alquiler en 2026, +10.000 EUR en 2027 y 2028

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014taHgH3F2aAsJapvbknJ6e
</commit_message>
<xml_diff>
--- a/finanzas/Prevision_2026_2028_prudente.xlsx
+++ b/finanzas/Prevision_2026_2028_prudente.xlsx
@@ -572,7 +572,7 @@
         <v>-91559.58</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>-109871.5</v>
+        <v>-91559.58</v>
       </c>
     </row>
     <row r="9">
@@ -585,13 +585,13 @@
         <v>-45022.32</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>-30874.84</v>
+        <v>-35874.84</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>-37049.81</v>
+        <v>-47049.81</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>-44459.77</v>
+        <v>-54459.77</v>
       </c>
     </row>
     <row r="10">
@@ -661,13 +661,13 @@
         <v>56474.66</v>
       </c>
       <c r="C13" s="8" t="n">
-        <v>216830.99</v>
+        <v>211830.99</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>262461.99</v>
+        <v>252461.99</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>317219.19</v>
+        <v>325531.11</v>
       </c>
     </row>
     <row r="14">
@@ -699,13 +699,13 @@
         <v>52522.61</v>
       </c>
       <c r="C15" s="8" t="n">
-        <v>213993.03</v>
+        <v>208993.03</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>259624.03</v>
+        <v>249624.03</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>314381.23</v>
+        <v>322693.15</v>
       </c>
     </row>
     <row r="16">
@@ -718,13 +718,13 @@
         <v>0</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>-43938.54</v>
+        <v>-42888.54</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>-50424.81</v>
+        <v>-48424.81</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>-61376.25</v>
+        <v>-63038.63</v>
       </c>
     </row>
     <row r="17">
@@ -737,13 +737,13 @@
         <v>52522.61</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>170054.49</v>
+        <v>166104.49</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>209199.23</v>
+        <v>201199.23</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>253004.99</v>
+        <v>259654.52</v>
       </c>
     </row>
     <row r="19">
@@ -913,13 +913,13 @@
         <v>64061.4</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>195964.33</v>
+        <v>192014.33</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>403704.11</v>
+        <v>391754.11</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>652692.96</v>
+        <v>647392.5</v>
       </c>
     </row>
     <row r="11">
@@ -932,13 +932,13 @@
         <v>199949.51</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>368677.63</v>
+        <v>364727.63</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>587439.74</v>
+        <v>575489.74</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>851920.1800000001</v>
+        <v>846619.72</v>
       </c>
     </row>
     <row r="13">
@@ -984,10 +984,10 @@
         <v>38033.68</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>208088.17</v>
+        <v>204138.17</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>417287.4</v>
+        <v>405337.4</v>
       </c>
     </row>
     <row r="16">
@@ -1000,13 +1000,13 @@
         <v>52522.61</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>170054.49</v>
+        <v>166104.49</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>209199.23</v>
+        <v>201199.23</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>253004.99</v>
+        <v>259654.52</v>
       </c>
     </row>
     <row r="17">
@@ -1038,13 +1038,13 @@
         <v>65373.68</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>235428.17</v>
+        <v>231478.17</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>444627.4</v>
+        <v>432677.4</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>697632.39</v>
+        <v>692331.92</v>
       </c>
     </row>
     <row r="19">
@@ -1163,13 +1163,13 @@
         <v>199949.51</v>
       </c>
       <c r="C25" s="8" t="n">
-        <v>368677.63</v>
+        <v>364727.63</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>587439.74</v>
+        <v>575489.74</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>851920.1800000001</v>
+        <v>846619.72</v>
       </c>
     </row>
   </sheetData>
@@ -1183,7 +1183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1229,14 +1229,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3. GASTOS DE PERSONAL: el coste anualizado de 2026 (61.039,72 €) se incrementa un 25%, hasta 76.299,65 €</t>
+          <t>3. GASTOS DE PERSONAL: el coste anualizado de 2026 (61.039,72 €) se incrementa un 25%, hasta 76.299,65 €.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (22,75% s/ventas). Ese peso sobre ventas se mantiene en 2027 y 2028.</t>
+          <t xml:space="preserve">   Para 2027 se incrementa un 20% sobre 2026 (91.559,58 €) y en 2028 se mantiene ese mismo nivel.</t>
         </is>
       </c>
     </row>
@@ -1246,60 +1246,67 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>4. OTROS GASTOS DE EXPLOTACIÓN: mantienen el peso observado en 2026 (9,21% s/ventas). Amortización constante</t>
+          <t>4. OTROS GASTOS DE EXPLOTACIÓN: mantienen el peso observado en 2026 (9,21% s/ventas) más un incremento del gasto</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (11.324,02 €/año, sin nuevas inversiones) y gastos financieros constantes (2.837,96 €/año). No se proyectan</t>
+          <t xml:space="preserve">   de alquiler de 5.000 € en 2026 y de 10.000 € anuales en 2027 y 2028. Amortización constante (11.324,02 €/año,</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   partidas no recurrentes de 2025 (deterioros, otros ingresos de explotación).</t>
+          <t xml:space="preserve">   sin nuevas inversiones) y gastos financieros constantes (2.837,96 €/año). No se proyectan partidas no</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   recurrentes de 2025 (deterioros, otros ingresos de explotación).</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>5. IMPUESTO SOBRE SOCIEDADES: tipos de microempresa (cifra de negocios &lt; 1M€, Ley 7/2024): 2026: 19%/21%;</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>5. IMPUESTO SOBRE SOCIEDADES: tipos de microempresa (cifra de negocios &lt; 1M€, Ley 7/2024): 2026: 19%/21%;</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t xml:space="preserve">   2027-2028: 17%/20% (primeros 50.000 € / resto). Sin compensación de bases imponibles negativas (criterio prudente).</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>6. BALANCE PREVISIONAL: clientes y acreedores comerciales crecen al ritmo de las ventas; el inmovilizado se reduce</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   por la amortización; la deuda financiera se mantiene constante; los resultados se traspasan a reservas al</t>
+          <t>6. BALANCE PREVISIONAL: clientes y acreedores comerciales crecen al ritmo de las ventas; el inmovilizado se reduce</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   por la amortización; la deuda financiera se mantiene constante; los resultados se traspasan a reservas al</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t xml:space="preserve">   ejercicio siguiente; el efectivo es la partida de cuadre (tesorería generada antes de dividendos o inversiones).</t>
         </is>

</xml_diff>

<commit_message>
Recalcular personal sobre base 2025: +25% en 2026, +20% en 2027-28
Personal 2026 = 97.251,95 x 1,25 = 121.564,94 EUR;
2027 y 2028 = 145.877,93 EUR (nivel 2026 +20%)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014taHgH3F2aAsJapvbknJ6e
</commit_message>
<xml_diff>
--- a/finanzas/Prevision_2026_2028_prudente.xlsx
+++ b/finanzas/Prevision_2026_2028_prudente.xlsx
@@ -566,13 +566,13 @@
         <v>-97251.95</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>-76299.64999999999</v>
+        <v>-121564.94</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>-91559.58</v>
+        <v>-145877.92</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>-91559.58</v>
+        <v>-145877.92</v>
       </c>
     </row>
     <row r="9">
@@ -661,13 +661,13 @@
         <v>56474.66</v>
       </c>
       <c r="C13" s="8" t="n">
-        <v>211830.99</v>
+        <v>166565.7</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>252461.99</v>
+        <v>198143.65</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>325531.11</v>
+        <v>271212.77</v>
       </c>
     </row>
     <row r="14">
@@ -699,13 +699,13 @@
         <v>52522.61</v>
       </c>
       <c r="C15" s="8" t="n">
-        <v>208993.03</v>
+        <v>163727.74</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>249624.03</v>
+        <v>195305.69</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>322693.15</v>
+        <v>268374.81</v>
       </c>
     </row>
     <row r="16">
@@ -718,13 +718,13 @@
         <v>0</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>-42888.54</v>
+        <v>-33382.83</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>-48424.81</v>
+        <v>-37561.14</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>-63038.63</v>
+        <v>-52174.96</v>
       </c>
     </row>
     <row r="17">
@@ -737,13 +737,13 @@
         <v>52522.61</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>166104.49</v>
+        <v>130344.92</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>201199.23</v>
+        <v>157744.55</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>259654.52</v>
+        <v>216199.84</v>
       </c>
     </row>
     <row r="19">
@@ -913,13 +913,13 @@
         <v>64061.4</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>192014.33</v>
+        <v>156254.75</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>391754.11</v>
+        <v>312539.86</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>647392.5</v>
+        <v>524723.5699999999</v>
       </c>
     </row>
     <row r="11">
@@ -932,13 +932,13 @@
         <v>199949.51</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>364727.63</v>
+        <v>328968.05</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>575489.74</v>
+        <v>496275.48</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>846619.72</v>
+        <v>723950.79</v>
       </c>
     </row>
     <row r="13">
@@ -984,10 +984,10 @@
         <v>38033.68</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>204138.17</v>
+        <v>168378.6</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>405337.4</v>
+        <v>326123.15</v>
       </c>
     </row>
     <row r="16">
@@ -1000,13 +1000,13 @@
         <v>52522.61</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>166104.49</v>
+        <v>130344.92</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>201199.23</v>
+        <v>157744.55</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>259654.52</v>
+        <v>216199.84</v>
       </c>
     </row>
     <row r="17">
@@ -1038,13 +1038,13 @@
         <v>65373.68</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>231478.17</v>
+        <v>195718.6</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>432677.4</v>
+        <v>353463.15</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>692331.92</v>
+        <v>569662.99</v>
       </c>
     </row>
     <row r="19">
@@ -1163,13 +1163,13 @@
         <v>199949.51</v>
       </c>
       <c r="C25" s="8" t="n">
-        <v>364727.63</v>
+        <v>328968.05</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>575489.74</v>
+        <v>496275.48</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>846619.72</v>
+        <v>723950.79</v>
       </c>
     </row>
   </sheetData>
@@ -1183,7 +1183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1229,84 +1229,91 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3. GASTOS DE PERSONAL: el coste anualizado de 2026 (61.039,72 €) se incrementa un 25%, hasta 76.299,65 €.</t>
+          <t>3. GASTOS DE PERSONAL: sobre el gasto real de 2025 (97.251,95 €) se aplica un incremento del 25% en 2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Para 2027 se incrementa un 20% sobre 2026 (91.559,58 €) y en 2028 se mantiene ese mismo nivel.</t>
+          <t xml:space="preserve">   (121.564,94 €). Para 2027 se incrementa un 20% adicional sobre 2026 (145.877,93 €) y en 2028 se mantiene</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ese mismo nivel.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>4. OTROS GASTOS DE EXPLOTACIÓN: mantienen el peso observado en 2026 (9,21% s/ventas) más un incremento del gasto</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   de alquiler de 5.000 € en 2026 y de 10.000 € anuales en 2027 y 2028. Amortización constante (11.324,02 €/año,</t>
+          <t>4. OTROS GASTOS DE EXPLOTACIÓN: mantienen el peso observado en 2026 (9,21% s/ventas) más un incremento del gasto</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   sin nuevas inversiones) y gastos financieros constantes (2.837,96 €/año). No se proyectan partidas no</t>
+          <t xml:space="preserve">   de alquiler de 5.000 € en 2026 y de 10.000 € anuales en 2027 y 2028. Amortización constante (11.324,02 €/año,</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t xml:space="preserve">   sin nuevas inversiones) y gastos financieros constantes (2.837,96 €/año). No se proyectan partidas no</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t xml:space="preserve">   recurrentes de 2025 (deterioros, otros ingresos de explotación).</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>5. IMPUESTO SOBRE SOCIEDADES: tipos de microempresa (cifra de negocios &lt; 1M€, Ley 7/2024): 2026: 19%/21%;</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>5. IMPUESTO SOBRE SOCIEDADES: tipos de microempresa (cifra de negocios &lt; 1M€, Ley 7/2024): 2026: 19%/21%;</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t xml:space="preserve">   2027-2028: 17%/20% (primeros 50.000 € / resto). Sin compensación de bases imponibles negativas (criterio prudente).</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-    </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>6. BALANCE PREVISIONAL: clientes y acreedores comerciales crecen al ritmo de las ventas; el inmovilizado se reduce</t>
-        </is>
-      </c>
+      <c r="A19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">   por la amortización; la deuda financiera se mantiene constante; los resultados se traspasan a reservas al</t>
+          <t>6. BALANCE PREVISIONAL: clientes y acreedores comerciales crecen al ritmo de las ventas; el inmovilizado se reduce</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   por la amortización; la deuda financiera se mantiene constante; los resultados se traspasan a reservas al</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t xml:space="preserve">   ejercicio siguiente; el efectivo es la partida de cuadre (tesorería generada antes de dividendos o inversiones).</t>
         </is>

</xml_diff>